<commit_message>
Group A foundation Done
</commit_message>
<xml_diff>
--- a/docs/Phase1_Sprint1_LeadCapture_Tracker.xlsx
+++ b/docs/Phase1_Sprint1_LeadCapture_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MEETCS_PROJECTS\AICRM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F65510-BF39-44F1-B2BC-7947C41E74D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF1E054-0009-4CC7-A518-1F8A7B646942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{E4894D6A-8C7A-4F10-BC2D-F6FD50435482}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E4894D6A-8C7A-4F10-BC2D-F6FD50435482}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>
@@ -1338,6 +1338,7 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>